<commit_message>
Updated the sheet with new entries.
</commit_message>
<xml_diff>
--- a/12600717.xlsx
+++ b/12600717.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python CAP776 Excell\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{578502CE-C951-4027-96BE-047FE141D52A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A72EA18-389E-4D17-94F4-42E6120596DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="74">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -245,6 +245,18 @@
   </si>
   <si>
     <t>No classes; dedicated day to recovery, project coding, and leisure.</t>
+  </si>
+  <si>
+    <t>Relaxed</t>
+  </si>
+  <si>
+    <t>Highly Satisfied</t>
+  </si>
+  <si>
+    <t>Sunday break; reviewed weak concepts and prepared schedule for upcoming week.</t>
+  </si>
+  <si>
+    <t>Attended 5 classes; started week with solid momentum and evening coding session.</t>
   </si>
 </sst>
 </file>
@@ -1299,49 +1311,97 @@
         <v>69</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+    <row r="12" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="8">
+        <v>46264</v>
+      </c>
+      <c r="B12" s="9">
+        <v>510</v>
+      </c>
+      <c r="C12" s="9">
+        <v>45</v>
+      </c>
+      <c r="D12" s="9">
+        <v>180</v>
+      </c>
+      <c r="E12" s="9">
+        <v>120</v>
+      </c>
+      <c r="F12" s="9">
+        <v>0</v>
+      </c>
+      <c r="G12" s="9">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9">
+        <v>270</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>1125</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+        <v>315</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="M12" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="N12" s="12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="8">
+        <v>46265</v>
+      </c>
+      <c r="B13" s="9">
+        <v>420</v>
+      </c>
+      <c r="C13" s="9">
+        <v>45</v>
+      </c>
+      <c r="D13" s="9">
+        <v>120</v>
+      </c>
+      <c r="E13" s="9">
+        <v>90</v>
+      </c>
+      <c r="F13" s="9">
+        <v>250</v>
+      </c>
+      <c r="G13" s="9">
+        <v>5</v>
+      </c>
+      <c r="H13" s="9">
+        <v>180</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>1105</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
+        <v>335</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="N13" s="12" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>

</xml_diff>

<commit_message>
updated the activity log
</commit_message>
<xml_diff>
--- a/12600717.xlsx
+++ b/12600717.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python CAP776 Excell\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78537C9F-F46D-4F5D-B4D0-4457E40F5560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3784CD57-9F51-4A86-B424-85A095B5F66C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -307,27 +307,6 @@
     <t>End of the week with 7 classes; completed weekly deliverables and lab write-ups.</t>
   </si>
   <si>
-    <t>Attended 6 classes; reviewed semester syllabus and organized study environment.</t>
-  </si>
-  <si>
-    <t>Heavy 7-class schedule; finished day with brief coding practice.</t>
-  </si>
-  <si>
-    <t>Weekend self-study; focused on full-stack architecture revision.</t>
-  </si>
-  <si>
-    <t>Sunday rest and reset; planned study goals for the upcoming week.</t>
-  </si>
-  <si>
-    <t>Attended 5 classes; productive evening study session.</t>
-  </si>
-  <si>
-    <t>Attended 5 classes; completed lab assignments efficiently.</t>
-  </si>
-  <si>
-    <t>Lighter schedule with 4 classes; focused on workout and course revision.</t>
-  </si>
-  <si>
     <t>Attended 6 classes; completed reading assignments in evening.</t>
   </si>
   <si>
@@ -365,6 +344,27 @@
   </si>
   <si>
     <t>AUGUST | SEPTEMBER</t>
+  </si>
+  <si>
+    <t>Saturday coding deep dive; completed full-stack microservice integration and API endpoints.</t>
+  </si>
+  <si>
+    <t>Sunday rest day; catch-up reading, weekly schedule review, and project planning.</t>
+  </si>
+  <si>
+    <t>Attended 5 classes; productive week start with evening competitive programming practice.</t>
+  </si>
+  <si>
+    <t>Attended 5 classes; finished lab exercises and prepared data science notes.</t>
+  </si>
+  <si>
+    <t>Lighter 4-class schedule; completed workout and revised core database concepts.</t>
+  </si>
+  <si>
+    <t>Attended 6 classes; focused during long lectures and worked on assignment submission.</t>
+  </si>
+  <si>
+    <t>End of academic week with 7 classes; finished weekly project deliverables and lab tasks.</t>
   </si>
 </sst>
 </file>
@@ -1022,7 +1022,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N419"/>
+  <dimension ref="A1:N412"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1059,7 +1059,7 @@
         <v>30</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
@@ -1084,7 +1084,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="G3" s="20"/>
     </row>
@@ -1150,9 +1150,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
-        <v>46240</v>
+        <v>46247</v>
       </c>
       <c r="B6" s="9">
         <v>450</v>
@@ -1161,7 +1161,7 @@
         <v>30</v>
       </c>
       <c r="D6" s="9">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="E6" s="9">
         <v>90</v>
@@ -1173,21 +1173,21 @@
         <v>6</v>
       </c>
       <c r="H6" s="9">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="I6" s="14">
-        <f t="shared" ref="I6:I21" si="0">IF(SUM(B6:F6,H6)=0,"",SUM(B6:F6,H6))</f>
+        <f t="shared" ref="I6:I14" si="0">IF(SUM(B6:F6,H6)=0,"",SUM(B6:F6,H6))</f>
         <v>1170</v>
       </c>
       <c r="J6" s="14">
-        <f t="shared" ref="J6:J24" si="1">IF(I6="","",1440-I6)</f>
+        <f t="shared" ref="J6:J17" si="1">IF(I6="","",1440-I6)</f>
         <v>270</v>
       </c>
       <c r="K6" s="10" t="s">
         <v>56</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="M6" s="10" t="s">
         <v>51</v>
@@ -1198,7 +1198,7 @@
     </row>
     <row r="7" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
-        <v>46241</v>
+        <v>46248</v>
       </c>
       <c r="B7" s="9">
         <v>420</v>
@@ -1233,7 +1233,7 @@
         <v>60</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>58</v>
@@ -1244,7 +1244,7 @@
     </row>
     <row r="8" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
-        <v>46242</v>
+        <v>46249</v>
       </c>
       <c r="B8" s="9">
         <v>510</v>
@@ -1288,9 +1288,9 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
-        <v>46243</v>
+        <v>46250</v>
       </c>
       <c r="B9" s="9">
         <v>480</v>
@@ -1334,9 +1334,9 @@
         <v>93</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="B10" s="9">
         <v>420</v>
@@ -1382,7 +1382,7 @@
     </row>
     <row r="11" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="B11" s="9">
         <v>450</v>
@@ -1428,7 +1428,7 @@
     </row>
     <row r="12" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
-        <v>46246</v>
+        <v>46253</v>
       </c>
       <c r="B12" s="9">
         <v>420</v>
@@ -1472,9 +1472,9 @@
         <v>96</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
-        <v>46247</v>
+        <v>46254</v>
       </c>
       <c r="B13" s="9">
         <v>450</v>
@@ -1520,7 +1520,7 @@
     </row>
     <row r="14" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
-        <v>46248</v>
+        <v>46255</v>
       </c>
       <c r="B14" s="9">
         <v>420</v>
@@ -1566,7 +1566,7 @@
     </row>
     <row r="15" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
-        <v>46249</v>
+        <v>46256</v>
       </c>
       <c r="B15" s="9">
         <v>510</v>
@@ -1590,7 +1590,7 @@
         <v>240</v>
       </c>
       <c r="I15" s="14">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="I15:I80" si="2">IF(SUM(B15:F15,H15)=0,"",SUM(B15:F15,H15))</f>
         <v>1140</v>
       </c>
       <c r="J15" s="14">
@@ -1610,9 +1610,9 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
-        <v>46250</v>
+        <v>46257</v>
       </c>
       <c r="B16" s="9">
         <v>480</v>
@@ -1636,7 +1636,7 @@
         <v>300</v>
       </c>
       <c r="I16" s="14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1095</v>
       </c>
       <c r="J16" s="14">
@@ -1656,9 +1656,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
-        <v>46251</v>
+        <v>46258</v>
       </c>
       <c r="B17" s="9">
         <v>420</v>
@@ -1682,7 +1682,7 @@
         <v>180</v>
       </c>
       <c r="I17" s="14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1105</v>
       </c>
       <c r="J17" s="14">
@@ -1699,12 +1699,12 @@
         <v>54</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>101</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="B18" s="9">
         <v>450</v>
@@ -1728,29 +1728,29 @@
         <v>150</v>
       </c>
       <c r="I18" s="14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1150</v>
       </c>
       <c r="J18" s="14">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="J18:J80" si="3">IF(I18="","",1440-I18)</f>
         <v>290</v>
       </c>
       <c r="K18" s="10" t="s">
         <v>55</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="M18" s="10" t="s">
         <v>54</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>102</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
-        <v>46253</v>
+        <v>46260</v>
       </c>
       <c r="B19" s="9">
         <v>420</v>
@@ -1759,7 +1759,7 @@
         <v>60</v>
       </c>
       <c r="D19" s="9">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="E19" s="9">
         <v>90</v>
@@ -1774,12 +1774,12 @@
         <v>180</v>
       </c>
       <c r="I19" s="14">
-        <f t="shared" si="0"/>
-        <v>1070</v>
+        <f t="shared" si="2"/>
+        <v>1040</v>
       </c>
       <c r="J19" s="14">
-        <f t="shared" si="1"/>
-        <v>370</v>
+        <f t="shared" si="3"/>
+        <v>400</v>
       </c>
       <c r="K19" s="10" t="s">
         <v>49</v>
@@ -1791,24 +1791,24 @@
         <v>51</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
-        <v>46254</v>
+        <v>46261</v>
       </c>
       <c r="B20" s="9">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="C20" s="9">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D20" s="9">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="E20" s="9">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F20" s="9">
         <v>300</v>
@@ -1817,15 +1817,15 @@
         <v>6</v>
       </c>
       <c r="H20" s="9">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="I20" s="14">
-        <f t="shared" si="0"/>
-        <v>1170</v>
+        <f t="shared" si="2"/>
+        <v>1215</v>
       </c>
       <c r="J20" s="14">
-        <f t="shared" si="1"/>
-        <v>270</v>
+        <f t="shared" si="3"/>
+        <v>225</v>
       </c>
       <c r="K20" s="10" t="s">
         <v>56</v>
@@ -1837,12 +1837,12 @@
         <v>51</v>
       </c>
       <c r="N20" s="11" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="B21" s="9">
         <v>420</v>
@@ -1851,10 +1851,10 @@
         <v>30</v>
       </c>
       <c r="D21" s="9">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="E21" s="9">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F21" s="9">
         <v>350</v>
@@ -1863,15 +1863,15 @@
         <v>7</v>
       </c>
       <c r="H21" s="9">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="I21" s="14">
-        <f t="shared" si="0"/>
-        <v>1190</v>
+        <f t="shared" si="2"/>
+        <v>1280</v>
       </c>
       <c r="J21" s="14">
-        <f t="shared" si="1"/>
-        <v>250</v>
+        <f t="shared" si="3"/>
+        <v>160</v>
       </c>
       <c r="K21" s="10" t="s">
         <v>60</v>
@@ -1883,24 +1883,24 @@
         <v>58</v>
       </c>
       <c r="N21" s="11" t="s">
-        <v>105</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
-        <v>46256</v>
+        <v>46263</v>
       </c>
       <c r="B22" s="9">
         <v>510</v>
       </c>
       <c r="C22" s="9">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D22" s="9">
+        <v>150</v>
+      </c>
+      <c r="E22" s="9">
         <v>180</v>
-      </c>
-      <c r="E22" s="9">
-        <v>150</v>
       </c>
       <c r="F22" s="9">
         <v>0</v>
@@ -1912,38 +1912,38 @@
         <v>240</v>
       </c>
       <c r="I22" s="14">
-        <f t="shared" ref="I22:I87" si="2">IF(SUM(B22:F22,H22)=0,"",SUM(B22:F22,H22))</f>
-        <v>1140</v>
+        <f t="shared" si="2"/>
+        <v>1130</v>
       </c>
       <c r="J22" s="14">
-        <f t="shared" si="1"/>
-        <v>300</v>
+        <f t="shared" si="3"/>
+        <v>310</v>
       </c>
       <c r="K22" s="10" t="s">
         <v>61</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="M22" s="10" t="s">
         <v>54</v>
       </c>
       <c r="N22" s="11" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="8">
-        <v>46257</v>
+        <v>46264</v>
       </c>
       <c r="B23" s="9">
-        <v>480</v>
+        <v>510</v>
       </c>
       <c r="C23" s="9">
         <v>45</v>
       </c>
       <c r="D23" s="9">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="E23" s="9">
         <v>120</v>
@@ -1955,32 +1955,32 @@
         <v>0</v>
       </c>
       <c r="H23" s="9">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="I23" s="14">
         <f t="shared" si="2"/>
-        <v>1095</v>
+        <v>1125</v>
       </c>
       <c r="J23" s="14">
-        <f t="shared" si="1"/>
-        <v>345</v>
+        <f t="shared" si="3"/>
+        <v>315</v>
       </c>
       <c r="K23" s="10" t="s">
         <v>68</v>
       </c>
       <c r="L23" s="10" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="M23" s="10" t="s">
         <v>54</v>
       </c>
       <c r="N23" s="11" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="8">
-        <v>46258</v>
+        <v>46265</v>
       </c>
       <c r="B24" s="9">
         <v>420</v>
@@ -2008,7 +2008,7 @@
         <v>1105</v>
       </c>
       <c r="J24" s="14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>335</v>
       </c>
       <c r="K24" s="10" t="s">
@@ -2021,12 +2021,12 @@
         <v>54</v>
       </c>
       <c r="N24" s="11" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A25" s="8">
-        <v>46259</v>
+        <v>46266</v>
       </c>
       <c r="B25" s="9">
         <v>450</v>
@@ -2054,34 +2054,34 @@
         <v>1150</v>
       </c>
       <c r="J25" s="14">
-        <f t="shared" ref="J25:J87" si="3">IF(I25="","",1440-I25)</f>
+        <f t="shared" si="3"/>
         <v>290</v>
       </c>
       <c r="K25" s="10" t="s">
         <v>55</v>
       </c>
       <c r="L25" s="10" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="M25" s="10" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="N25" s="11" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="8">
-        <v>46260</v>
+        <v>46267</v>
       </c>
       <c r="B26" s="9">
         <v>420</v>
       </c>
       <c r="C26" s="9">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="D26" s="9">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="E26" s="9">
         <v>90</v>
@@ -2097,11 +2097,11 @@
       </c>
       <c r="I26" s="14">
         <f t="shared" si="2"/>
-        <v>1040</v>
+        <v>1055</v>
       </c>
       <c r="J26" s="14">
         <f t="shared" si="3"/>
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="K26" s="10" t="s">
         <v>49</v>
@@ -2112,25 +2112,25 @@
       <c r="M26" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="N26" s="11" t="s">
-        <v>64</v>
+      <c r="N26" s="17" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="8">
-        <v>46261</v>
+        <v>46268</v>
       </c>
       <c r="B27" s="9">
-        <v>480</v>
+        <v>450</v>
       </c>
       <c r="C27" s="9">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D27" s="9">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="E27" s="9">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F27" s="9">
         <v>300</v>
@@ -2143,28 +2143,28 @@
       </c>
       <c r="I27" s="14">
         <f t="shared" si="2"/>
-        <v>1215</v>
+        <v>1170</v>
       </c>
       <c r="J27" s="14">
         <f t="shared" si="3"/>
-        <v>225</v>
+        <v>270</v>
       </c>
       <c r="K27" s="10" t="s">
         <v>56</v>
       </c>
       <c r="L27" s="10" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="M27" s="10" t="s">
         <v>51</v>
       </c>
       <c r="N27" s="11" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A28" s="8">
-        <v>46262</v>
+        <v>46269</v>
       </c>
       <c r="B28" s="9">
         <v>420</v>
@@ -2173,10 +2173,10 @@
         <v>30</v>
       </c>
       <c r="D28" s="9">
+        <v>90</v>
+      </c>
+      <c r="E28" s="9">
         <v>120</v>
-      </c>
-      <c r="E28" s="9">
-        <v>150</v>
       </c>
       <c r="F28" s="9">
         <v>350</v>
@@ -2185,44 +2185,44 @@
         <v>7</v>
       </c>
       <c r="H28" s="9">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="I28" s="14">
         <f t="shared" si="2"/>
-        <v>1280</v>
+        <v>1190</v>
       </c>
       <c r="J28" s="14">
         <f t="shared" si="3"/>
-        <v>160</v>
+        <v>250</v>
       </c>
       <c r="K28" s="10" t="s">
         <v>60</v>
       </c>
       <c r="L28" s="10" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="M28" s="10" t="s">
         <v>58</v>
       </c>
       <c r="N28" s="11" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A29" s="8">
-        <v>46263</v>
+        <v>46270</v>
       </c>
       <c r="B29" s="9">
         <v>510</v>
       </c>
       <c r="C29" s="9">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D29" s="9">
+        <v>180</v>
+      </c>
+      <c r="E29" s="9">
         <v>150</v>
-      </c>
-      <c r="E29" s="9">
-        <v>180</v>
       </c>
       <c r="F29" s="9">
         <v>0</v>
@@ -2235,37 +2235,37 @@
       </c>
       <c r="I29" s="14">
         <f t="shared" si="2"/>
-        <v>1130</v>
+        <v>1140</v>
       </c>
       <c r="J29" s="14">
         <f t="shared" si="3"/>
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="K29" s="10" t="s">
         <v>61</v>
       </c>
       <c r="L29" s="10" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="M29" s="10" t="s">
         <v>54</v>
       </c>
       <c r="N29" s="11" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A30" s="8">
-        <v>46264</v>
+        <v>46271</v>
       </c>
       <c r="B30" s="9">
-        <v>510</v>
+        <v>480</v>
       </c>
       <c r="C30" s="9">
         <v>45</v>
       </c>
       <c r="D30" s="9">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="E30" s="9">
         <v>120</v>
@@ -2277,32 +2277,32 @@
         <v>0</v>
       </c>
       <c r="H30" s="9">
-        <v>270</v>
+        <v>300</v>
       </c>
       <c r="I30" s="14">
         <f t="shared" si="2"/>
-        <v>1125</v>
+        <v>1095</v>
       </c>
       <c r="J30" s="14">
         <f t="shared" si="3"/>
-        <v>315</v>
+        <v>345</v>
       </c>
       <c r="K30" s="10" t="s">
         <v>68</v>
       </c>
       <c r="L30" s="10" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="M30" s="10" t="s">
         <v>54</v>
       </c>
       <c r="N30" s="11" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A31" s="8">
-        <v>46265</v>
+        <v>46272</v>
       </c>
       <c r="B31" s="9">
         <v>420</v>
@@ -2343,12 +2343,12 @@
         <v>54</v>
       </c>
       <c r="N31" s="11" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="8">
-        <v>46266</v>
+        <v>46273</v>
       </c>
       <c r="B32" s="9">
         <v>450</v>
@@ -2383,24 +2383,24 @@
         <v>55</v>
       </c>
       <c r="L32" s="10" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="M32" s="10" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="N32" s="11" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="8">
-        <v>46267</v>
+        <v>46274</v>
       </c>
       <c r="B33" s="9">
         <v>420</v>
       </c>
       <c r="C33" s="9">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D33" s="9">
         <v>120</v>
@@ -2419,11 +2419,11 @@
       </c>
       <c r="I33" s="14">
         <f t="shared" si="2"/>
-        <v>1055</v>
+        <v>1070</v>
       </c>
       <c r="J33" s="14">
         <f t="shared" si="3"/>
-        <v>385</v>
+        <v>370</v>
       </c>
       <c r="K33" s="10" t="s">
         <v>49</v>
@@ -2434,13 +2434,13 @@
       <c r="M33" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="N33" s="17" t="s">
-        <v>82</v>
+      <c r="N33" s="11" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="8">
-        <v>46268</v>
+        <v>46275</v>
       </c>
       <c r="B34" s="9">
         <v>450</v>
@@ -2449,7 +2449,7 @@
         <v>30</v>
       </c>
       <c r="D34" s="9">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="E34" s="9">
         <v>90</v>
@@ -2461,7 +2461,7 @@
         <v>6</v>
       </c>
       <c r="H34" s="9">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="I34" s="14">
         <f t="shared" si="2"/>
@@ -2475,18 +2475,18 @@
         <v>56</v>
       </c>
       <c r="L34" s="10" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="M34" s="10" t="s">
         <v>51</v>
       </c>
       <c r="N34" s="11" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A35" s="8">
-        <v>46269</v>
+        <v>46276</v>
       </c>
       <c r="B35" s="9">
         <v>420</v>
@@ -2521,18 +2521,18 @@
         <v>60</v>
       </c>
       <c r="L35" s="10" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="M35" s="10" t="s">
         <v>58</v>
       </c>
       <c r="N35" s="11" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="8">
-        <v>46270</v>
+        <v>46277</v>
       </c>
       <c r="B36" s="9">
         <v>510</v>
@@ -2573,12 +2573,12 @@
         <v>54</v>
       </c>
       <c r="N36" s="11" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A37" s="8">
-        <v>46271</v>
+        <v>46278</v>
       </c>
       <c r="B37" s="9">
         <v>480</v>
@@ -2619,12 +2619,12 @@
         <v>54</v>
       </c>
       <c r="N37" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A38" s="8">
-        <v>46272</v>
+        <v>46279</v>
       </c>
       <c r="B38" s="9">
         <v>420</v>
@@ -2665,12 +2665,12 @@
         <v>54</v>
       </c>
       <c r="N38" s="11" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A39" s="8">
-        <v>46273</v>
+        <v>46280</v>
       </c>
       <c r="B39" s="9">
         <v>450</v>
@@ -2711,12 +2711,12 @@
         <v>54</v>
       </c>
       <c r="N39" s="11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A40" s="8">
-        <v>46274</v>
+        <v>46281</v>
       </c>
       <c r="B40" s="9">
         <v>420</v>
@@ -2757,12 +2757,12 @@
         <v>51</v>
       </c>
       <c r="N40" s="11" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A41" s="8">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="B41" s="9">
         <v>450</v>
@@ -2803,12 +2803,12 @@
         <v>51</v>
       </c>
       <c r="N41" s="11" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A42" s="8">
-        <v>46276</v>
+        <v>46283</v>
       </c>
       <c r="B42" s="9">
         <v>420</v>
@@ -2849,12 +2849,12 @@
         <v>58</v>
       </c>
       <c r="N42" s="11" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A43" s="8">
-        <v>46277</v>
+        <v>46284</v>
       </c>
       <c r="B43" s="9">
         <v>510</v>
@@ -2895,12 +2895,12 @@
         <v>54</v>
       </c>
       <c r="N43" s="11" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A44" s="8">
-        <v>46278</v>
+        <v>46285</v>
       </c>
       <c r="B44" s="9">
         <v>480</v>
@@ -2941,12 +2941,12 @@
         <v>54</v>
       </c>
       <c r="N44" s="11" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A45" s="8">
-        <v>46279</v>
+        <v>46286</v>
       </c>
       <c r="B45" s="9">
         <v>420</v>
@@ -2987,12 +2987,12 @@
         <v>54</v>
       </c>
       <c r="N45" s="11" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="46" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A46" s="8">
-        <v>46280</v>
+        <v>46287</v>
       </c>
       <c r="B46" s="9">
         <v>450</v>
@@ -3033,12 +3033,12 @@
         <v>54</v>
       </c>
       <c r="N46" s="11" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A47" s="8">
-        <v>46281</v>
+        <v>46288</v>
       </c>
       <c r="B47" s="9">
         <v>420</v>
@@ -3079,12 +3079,12 @@
         <v>51</v>
       </c>
       <c r="N47" s="11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="48" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A48" s="8">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="B48" s="9">
         <v>450</v>
@@ -3125,12 +3125,12 @@
         <v>51</v>
       </c>
       <c r="N48" s="11" t="s">
-        <v>88</v>
+        <v>108</v>
       </c>
     </row>
     <row r="49" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A49" s="8">
-        <v>46283</v>
+        <v>46290</v>
       </c>
       <c r="B49" s="9">
         <v>420</v>
@@ -3171,7 +3171,7 @@
         <v>58</v>
       </c>
       <c r="N49" s="11" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
@@ -3866,11 +3866,11 @@
       <c r="G81" s="9"/>
       <c r="H81" s="9"/>
       <c r="I81" s="14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="I81:I144" si="4">IF(SUM(B81:F81,H81)=0,"",SUM(B81:F81,H81))</f>
         <v/>
       </c>
       <c r="J81" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="J81:J144" si="5">IF(I81="","",1440-I81)</f>
         <v/>
       </c>
       <c r="K81" s="10"/>
@@ -3888,11 +3888,11 @@
       <c r="G82" s="9"/>
       <c r="H82" s="9"/>
       <c r="I82" s="14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J82" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K82" s="10"/>
@@ -3910,11 +3910,11 @@
       <c r="G83" s="9"/>
       <c r="H83" s="9"/>
       <c r="I83" s="14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J83" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K83" s="10"/>
@@ -3932,11 +3932,11 @@
       <c r="G84" s="9"/>
       <c r="H84" s="9"/>
       <c r="I84" s="14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J84" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K84" s="10"/>
@@ -3954,11 +3954,11 @@
       <c r="G85" s="9"/>
       <c r="H85" s="9"/>
       <c r="I85" s="14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J85" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K85" s="10"/>
@@ -3976,11 +3976,11 @@
       <c r="G86" s="9"/>
       <c r="H86" s="9"/>
       <c r="I86" s="14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J86" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K86" s="10"/>
@@ -3998,11 +3998,11 @@
       <c r="G87" s="9"/>
       <c r="H87" s="9"/>
       <c r="I87" s="14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J87" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K87" s="10"/>
@@ -4020,11 +4020,11 @@
       <c r="G88" s="9"/>
       <c r="H88" s="9"/>
       <c r="I88" s="14" t="str">
-        <f t="shared" ref="I88:I151" si="4">IF(SUM(B88:F88,H88)=0,"",SUM(B88:F88,H88))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J88" s="14" t="str">
-        <f t="shared" ref="J88:J151" si="5">IF(I88="","",1440-I88)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K88" s="10"/>
@@ -5274,11 +5274,11 @@
       <c r="G145" s="9"/>
       <c r="H145" s="9"/>
       <c r="I145" s="14" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I145:I208" si="6">IF(SUM(B145:F145,H145)=0,"",SUM(B145:F145,H145))</f>
         <v/>
       </c>
       <c r="J145" s="14" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="J145:J208" si="7">IF(I145="","",1440-I145)</f>
         <v/>
       </c>
       <c r="K145" s="10"/>
@@ -5296,11 +5296,11 @@
       <c r="G146" s="9"/>
       <c r="H146" s="9"/>
       <c r="I146" s="14" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J146" s="14" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K146" s="10"/>
@@ -5310,19 +5310,19 @@
     </row>
     <row r="147" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A147" s="8"/>
-      <c r="B147" s="9"/>
-      <c r="C147" s="9"/>
-      <c r="D147" s="9"/>
-      <c r="E147" s="9"/>
-      <c r="F147" s="9"/>
-      <c r="G147" s="9"/>
+      <c r="B147" s="13"/>
+      <c r="C147" s="13"/>
+      <c r="D147" s="13"/>
+      <c r="E147" s="13"/>
+      <c r="F147" s="13"/>
+      <c r="G147" s="13"/>
       <c r="H147" s="9"/>
       <c r="I147" s="14" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J147" s="14" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K147" s="10"/>
@@ -5332,123 +5332,123 @@
     </row>
     <row r="148" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A148" s="8"/>
-      <c r="B148" s="9"/>
-      <c r="C148" s="9"/>
-      <c r="D148" s="9"/>
-      <c r="E148" s="9"/>
-      <c r="F148" s="9"/>
-      <c r="G148" s="9"/>
-      <c r="H148" s="9"/>
+      <c r="B148" s="13"/>
+      <c r="C148" s="13"/>
+      <c r="D148" s="13"/>
+      <c r="E148" s="13"/>
+      <c r="F148" s="13"/>
+      <c r="G148" s="13"/>
+      <c r="H148" s="13"/>
       <c r="I148" s="14" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J148" s="14" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K148" s="10"/>
-      <c r="L148" s="10"/>
-      <c r="M148" s="10"/>
-      <c r="N148" s="11"/>
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="K148" s="15"/>
+      <c r="L148" s="15"/>
+      <c r="M148" s="15"/>
+      <c r="N148" s="16"/>
     </row>
     <row r="149" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A149" s="8"/>
-      <c r="B149" s="9"/>
-      <c r="C149" s="9"/>
-      <c r="D149" s="9"/>
-      <c r="E149" s="9"/>
-      <c r="F149" s="9"/>
-      <c r="G149" s="9"/>
-      <c r="H149" s="9"/>
+      <c r="B149" s="13"/>
+      <c r="C149" s="13"/>
+      <c r="D149" s="13"/>
+      <c r="E149" s="13"/>
+      <c r="F149" s="13"/>
+      <c r="G149" s="13"/>
+      <c r="H149" s="13"/>
       <c r="I149" s="14" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J149" s="14" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K149" s="10"/>
-      <c r="L149" s="10"/>
-      <c r="M149" s="10"/>
-      <c r="N149" s="11"/>
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="K149" s="15"/>
+      <c r="L149" s="15"/>
+      <c r="M149" s="15"/>
+      <c r="N149" s="16"/>
     </row>
     <row r="150" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A150" s="8"/>
-      <c r="B150" s="9"/>
-      <c r="C150" s="9"/>
-      <c r="D150" s="9"/>
-      <c r="E150" s="9"/>
-      <c r="F150" s="9"/>
-      <c r="G150" s="9"/>
-      <c r="H150" s="9"/>
+      <c r="B150" s="13"/>
+      <c r="C150" s="13"/>
+      <c r="D150" s="13"/>
+      <c r="E150" s="13"/>
+      <c r="F150" s="13"/>
+      <c r="G150" s="13"/>
+      <c r="H150" s="13"/>
       <c r="I150" s="14" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J150" s="14" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K150" s="10"/>
-      <c r="L150" s="10"/>
-      <c r="M150" s="10"/>
-      <c r="N150" s="11"/>
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="K150" s="15"/>
+      <c r="L150" s="15"/>
+      <c r="M150" s="15"/>
+      <c r="N150" s="16"/>
     </row>
     <row r="151" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A151" s="8"/>
-      <c r="B151" s="9"/>
-      <c r="C151" s="9"/>
-      <c r="D151" s="9"/>
-      <c r="E151" s="9"/>
-      <c r="F151" s="9"/>
-      <c r="G151" s="9"/>
-      <c r="H151" s="9"/>
+      <c r="B151" s="13"/>
+      <c r="C151" s="13"/>
+      <c r="D151" s="13"/>
+      <c r="E151" s="13"/>
+      <c r="F151" s="13"/>
+      <c r="G151" s="13"/>
+      <c r="H151" s="13"/>
       <c r="I151" s="14" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J151" s="14" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K151" s="10"/>
-      <c r="L151" s="10"/>
-      <c r="M151" s="10"/>
-      <c r="N151" s="11"/>
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="K151" s="15"/>
+      <c r="L151" s="15"/>
+      <c r="M151" s="15"/>
+      <c r="N151" s="16"/>
     </row>
     <row r="152" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A152" s="8"/>
-      <c r="B152" s="9"/>
-      <c r="C152" s="9"/>
-      <c r="D152" s="9"/>
-      <c r="E152" s="9"/>
-      <c r="F152" s="9"/>
-      <c r="G152" s="9"/>
-      <c r="H152" s="9"/>
+      <c r="B152" s="13"/>
+      <c r="C152" s="13"/>
+      <c r="D152" s="13"/>
+      <c r="E152" s="13"/>
+      <c r="F152" s="13"/>
+      <c r="G152" s="13"/>
+      <c r="H152" s="13"/>
       <c r="I152" s="14" t="str">
-        <f t="shared" ref="I152:I215" si="6">IF(SUM(B152:F152,H152)=0,"",SUM(B152:F152,H152))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J152" s="14" t="str">
-        <f t="shared" ref="J152:J215" si="7">IF(I152="","",1440-I152)</f>
-        <v/>
-      </c>
-      <c r="K152" s="10"/>
-      <c r="L152" s="10"/>
-      <c r="M152" s="10"/>
-      <c r="N152" s="11"/>
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="K152" s="15"/>
+      <c r="L152" s="15"/>
+      <c r="M152" s="15"/>
+      <c r="N152" s="16"/>
     </row>
     <row r="153" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A153" s="8"/>
-      <c r="B153" s="9"/>
-      <c r="C153" s="9"/>
-      <c r="D153" s="9"/>
-      <c r="E153" s="9"/>
-      <c r="F153" s="9"/>
-      <c r="G153" s="9"/>
-      <c r="H153" s="9"/>
+      <c r="B153" s="13"/>
+      <c r="C153" s="13"/>
+      <c r="D153" s="13"/>
+      <c r="E153" s="13"/>
+      <c r="F153" s="13"/>
+      <c r="G153" s="13"/>
+      <c r="H153" s="13"/>
       <c r="I153" s="14" t="str">
         <f t="shared" si="6"/>
         <v/>
@@ -5457,10 +5457,10 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K153" s="10"/>
-      <c r="L153" s="10"/>
-      <c r="M153" s="10"/>
-      <c r="N153" s="11"/>
+      <c r="K153" s="15"/>
+      <c r="L153" s="15"/>
+      <c r="M153" s="15"/>
+      <c r="N153" s="16"/>
     </row>
     <row r="154" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A154" s="8"/>
@@ -5470,7 +5470,7 @@
       <c r="E154" s="13"/>
       <c r="F154" s="13"/>
       <c r="G154" s="13"/>
-      <c r="H154" s="9"/>
+      <c r="H154" s="13"/>
       <c r="I154" s="14" t="str">
         <f t="shared" si="6"/>
         <v/>
@@ -5479,10 +5479,10 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="K154" s="10"/>
-      <c r="L154" s="10"/>
-      <c r="M154" s="10"/>
-      <c r="N154" s="11"/>
+      <c r="K154" s="15"/>
+      <c r="L154" s="15"/>
+      <c r="M154" s="15"/>
+      <c r="N154" s="16"/>
     </row>
     <row r="155" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A155" s="8"/>
@@ -6682,11 +6682,11 @@
       <c r="G209" s="13"/>
       <c r="H209" s="13"/>
       <c r="I209" s="14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="I209:I272" si="8">IF(SUM(B209:F209,H209)=0,"",SUM(B209:F209,H209))</f>
         <v/>
       </c>
       <c r="J209" s="14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="J209:J272" si="9">IF(I209="","",1440-I209)</f>
         <v/>
       </c>
       <c r="K209" s="15"/>
@@ -6704,11 +6704,11 @@
       <c r="G210" s="13"/>
       <c r="H210" s="13"/>
       <c r="I210" s="14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J210" s="14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K210" s="15"/>
@@ -6726,11 +6726,11 @@
       <c r="G211" s="13"/>
       <c r="H211" s="13"/>
       <c r="I211" s="14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J211" s="14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K211" s="15"/>
@@ -6748,11 +6748,11 @@
       <c r="G212" s="13"/>
       <c r="H212" s="13"/>
       <c r="I212" s="14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J212" s="14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K212" s="15"/>
@@ -6770,11 +6770,11 @@
       <c r="G213" s="13"/>
       <c r="H213" s="13"/>
       <c r="I213" s="14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J213" s="14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K213" s="15"/>
@@ -6792,11 +6792,11 @@
       <c r="G214" s="13"/>
       <c r="H214" s="13"/>
       <c r="I214" s="14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J214" s="14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K214" s="15"/>
@@ -6814,11 +6814,11 @@
       <c r="G215" s="13"/>
       <c r="H215" s="13"/>
       <c r="I215" s="14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J215" s="14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K215" s="15"/>
@@ -6836,11 +6836,11 @@
       <c r="G216" s="13"/>
       <c r="H216" s="13"/>
       <c r="I216" s="14" t="str">
-        <f t="shared" ref="I216:I279" si="8">IF(SUM(B216:F216,H216)=0,"",SUM(B216:F216,H216))</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J216" s="14" t="str">
-        <f t="shared" ref="J216:J279" si="9">IF(I216="","",1440-I216)</f>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K216" s="15"/>
@@ -6981,7 +6981,7 @@
       <c r="N222" s="16"/>
     </row>
     <row r="223" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A223" s="8"/>
+      <c r="A223" s="12"/>
       <c r="B223" s="13"/>
       <c r="C223" s="13"/>
       <c r="D223" s="13"/>
@@ -7003,7 +7003,7 @@
       <c r="N223" s="16"/>
     </row>
     <row r="224" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A224" s="8"/>
+      <c r="A224" s="12"/>
       <c r="B224" s="13"/>
       <c r="C224" s="13"/>
       <c r="D224" s="13"/>
@@ -7025,7 +7025,7 @@
       <c r="N224" s="16"/>
     </row>
     <row r="225" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A225" s="8"/>
+      <c r="A225" s="12"/>
       <c r="B225" s="13"/>
       <c r="C225" s="13"/>
       <c r="D225" s="13"/>
@@ -7047,7 +7047,7 @@
       <c r="N225" s="16"/>
     </row>
     <row r="226" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A226" s="8"/>
+      <c r="A226" s="12"/>
       <c r="B226" s="13"/>
       <c r="C226" s="13"/>
       <c r="D226" s="13"/>
@@ -7069,7 +7069,7 @@
       <c r="N226" s="16"/>
     </row>
     <row r="227" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A227" s="8"/>
+      <c r="A227" s="12"/>
       <c r="B227" s="13"/>
       <c r="C227" s="13"/>
       <c r="D227" s="13"/>
@@ -7091,7 +7091,7 @@
       <c r="N227" s="16"/>
     </row>
     <row r="228" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A228" s="8"/>
+      <c r="A228" s="12"/>
       <c r="B228" s="13"/>
       <c r="C228" s="13"/>
       <c r="D228" s="13"/>
@@ -7113,7 +7113,7 @@
       <c r="N228" s="16"/>
     </row>
     <row r="229" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A229" s="8"/>
+      <c r="A229" s="12"/>
       <c r="B229" s="13"/>
       <c r="C229" s="13"/>
       <c r="D229" s="13"/>
@@ -8090,11 +8090,11 @@
       <c r="G273" s="13"/>
       <c r="H273" s="13"/>
       <c r="I273" s="14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="I273:I336" si="10">IF(SUM(B273:F273,H273)=0,"",SUM(B273:F273,H273))</f>
         <v/>
       </c>
       <c r="J273" s="14" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="J273:J336" si="11">IF(I273="","",1440-I273)</f>
         <v/>
       </c>
       <c r="K273" s="15"/>
@@ -8112,11 +8112,11 @@
       <c r="G274" s="13"/>
       <c r="H274" s="13"/>
       <c r="I274" s="14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J274" s="14" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K274" s="15"/>
@@ -8134,11 +8134,11 @@
       <c r="G275" s="13"/>
       <c r="H275" s="13"/>
       <c r="I275" s="14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J275" s="14" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K275" s="15"/>
@@ -8156,11 +8156,11 @@
       <c r="G276" s="13"/>
       <c r="H276" s="13"/>
       <c r="I276" s="14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J276" s="14" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K276" s="15"/>
@@ -8178,11 +8178,11 @@
       <c r="G277" s="13"/>
       <c r="H277" s="13"/>
       <c r="I277" s="14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J277" s="14" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K277" s="15"/>
@@ -8200,11 +8200,11 @@
       <c r="G278" s="13"/>
       <c r="H278" s="13"/>
       <c r="I278" s="14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J278" s="14" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K278" s="15"/>
@@ -8222,11 +8222,11 @@
       <c r="G279" s="13"/>
       <c r="H279" s="13"/>
       <c r="I279" s="14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J279" s="14" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K279" s="15"/>
@@ -8244,11 +8244,11 @@
       <c r="G280" s="13"/>
       <c r="H280" s="13"/>
       <c r="I280" s="14" t="str">
-        <f t="shared" ref="I280:I343" si="10">IF(SUM(B280:F280,H280)=0,"",SUM(B280:F280,H280))</f>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J280" s="14" t="str">
-        <f t="shared" ref="J280:J343" si="11">IF(I280="","",1440-I280)</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K280" s="15"/>
@@ -9498,11 +9498,11 @@
       <c r="G337" s="13"/>
       <c r="H337" s="13"/>
       <c r="I337" s="14" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I337:I400" si="12">IF(SUM(B337:F337,H337)=0,"",SUM(B337:F337,H337))</f>
         <v/>
       </c>
       <c r="J337" s="14" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="J337:J400" si="13">IF(I337="","",1440-I337)</f>
         <v/>
       </c>
       <c r="K337" s="15"/>
@@ -9520,11 +9520,11 @@
       <c r="G338" s="13"/>
       <c r="H338" s="13"/>
       <c r="I338" s="14" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J338" s="14" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K338" s="15"/>
@@ -9542,11 +9542,11 @@
       <c r="G339" s="13"/>
       <c r="H339" s="13"/>
       <c r="I339" s="14" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J339" s="14" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K339" s="15"/>
@@ -9564,11 +9564,11 @@
       <c r="G340" s="13"/>
       <c r="H340" s="13"/>
       <c r="I340" s="14" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J340" s="14" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K340" s="15"/>
@@ -9586,11 +9586,11 @@
       <c r="G341" s="13"/>
       <c r="H341" s="13"/>
       <c r="I341" s="14" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J341" s="14" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K341" s="15"/>
@@ -9608,11 +9608,11 @@
       <c r="G342" s="13"/>
       <c r="H342" s="13"/>
       <c r="I342" s="14" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J342" s="14" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K342" s="15"/>
@@ -9630,11 +9630,11 @@
       <c r="G343" s="13"/>
       <c r="H343" s="13"/>
       <c r="I343" s="14" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J343" s="14" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K343" s="15"/>
@@ -9652,11 +9652,11 @@
       <c r="G344" s="13"/>
       <c r="H344" s="13"/>
       <c r="I344" s="14" t="str">
-        <f t="shared" ref="I344:I407" si="12">IF(SUM(B344:F344,H344)=0,"",SUM(B344:F344,H344))</f>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J344" s="14" t="str">
-        <f t="shared" ref="J344:J407" si="13">IF(I344="","",1440-I344)</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="K344" s="15"/>
@@ -10906,11 +10906,11 @@
       <c r="G401" s="13"/>
       <c r="H401" s="13"/>
       <c r="I401" s="14" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="I401:I412" si="14">IF(SUM(B401:F401,H401)=0,"",SUM(B401:F401,H401))</f>
         <v/>
       </c>
       <c r="J401" s="14" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="J401:J412" si="15">IF(I401="","",1440-I401)</f>
         <v/>
       </c>
       <c r="K401" s="15"/>
@@ -10928,11 +10928,11 @@
       <c r="G402" s="13"/>
       <c r="H402" s="13"/>
       <c r="I402" s="14" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J402" s="14" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K402" s="15"/>
@@ -10950,11 +10950,11 @@
       <c r="G403" s="13"/>
       <c r="H403" s="13"/>
       <c r="I403" s="14" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J403" s="14" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K403" s="15"/>
@@ -10972,11 +10972,11 @@
       <c r="G404" s="13"/>
       <c r="H404" s="13"/>
       <c r="I404" s="14" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J404" s="14" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K404" s="15"/>
@@ -10994,11 +10994,11 @@
       <c r="G405" s="13"/>
       <c r="H405" s="13"/>
       <c r="I405" s="14" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J405" s="14" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K405" s="15"/>
@@ -11016,11 +11016,11 @@
       <c r="G406" s="13"/>
       <c r="H406" s="13"/>
       <c r="I406" s="14" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J406" s="14" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K406" s="15"/>
@@ -11038,11 +11038,11 @@
       <c r="G407" s="13"/>
       <c r="H407" s="13"/>
       <c r="I407" s="14" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J407" s="14" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K407" s="15"/>
@@ -11060,11 +11060,11 @@
       <c r="G408" s="13"/>
       <c r="H408" s="13"/>
       <c r="I408" s="14" t="str">
-        <f t="shared" ref="I408:I419" si="14">IF(SUM(B408:F408,H408)=0,"",SUM(B408:F408,H408))</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="J408" s="14" t="str">
-        <f t="shared" ref="J408:J419" si="15">IF(I408="","",1440-I408)</f>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="K408" s="15"/>
@@ -11160,160 +11160,6 @@
       <c r="M412" s="15"/>
       <c r="N412" s="16"/>
     </row>
-    <row r="413" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A413" s="12"/>
-      <c r="B413" s="13"/>
-      <c r="C413" s="13"/>
-      <c r="D413" s="13"/>
-      <c r="E413" s="13"/>
-      <c r="F413" s="13"/>
-      <c r="G413" s="13"/>
-      <c r="H413" s="13"/>
-      <c r="I413" s="14" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="J413" s="14" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="K413" s="15"/>
-      <c r="L413" s="15"/>
-      <c r="M413" s="15"/>
-      <c r="N413" s="16"/>
-    </row>
-    <row r="414" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A414" s="12"/>
-      <c r="B414" s="13"/>
-      <c r="C414" s="13"/>
-      <c r="D414" s="13"/>
-      <c r="E414" s="13"/>
-      <c r="F414" s="13"/>
-      <c r="G414" s="13"/>
-      <c r="H414" s="13"/>
-      <c r="I414" s="14" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="J414" s="14" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="K414" s="15"/>
-      <c r="L414" s="15"/>
-      <c r="M414" s="15"/>
-      <c r="N414" s="16"/>
-    </row>
-    <row r="415" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A415" s="12"/>
-      <c r="B415" s="13"/>
-      <c r="C415" s="13"/>
-      <c r="D415" s="13"/>
-      <c r="E415" s="13"/>
-      <c r="F415" s="13"/>
-      <c r="G415" s="13"/>
-      <c r="H415" s="13"/>
-      <c r="I415" s="14" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="J415" s="14" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="K415" s="15"/>
-      <c r="L415" s="15"/>
-      <c r="M415" s="15"/>
-      <c r="N415" s="16"/>
-    </row>
-    <row r="416" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A416" s="12"/>
-      <c r="B416" s="13"/>
-      <c r="C416" s="13"/>
-      <c r="D416" s="13"/>
-      <c r="E416" s="13"/>
-      <c r="F416" s="13"/>
-      <c r="G416" s="13"/>
-      <c r="H416" s="13"/>
-      <c r="I416" s="14" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="J416" s="14" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="K416" s="15"/>
-      <c r="L416" s="15"/>
-      <c r="M416" s="15"/>
-      <c r="N416" s="16"/>
-    </row>
-    <row r="417" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A417" s="12"/>
-      <c r="B417" s="13"/>
-      <c r="C417" s="13"/>
-      <c r="D417" s="13"/>
-      <c r="E417" s="13"/>
-      <c r="F417" s="13"/>
-      <c r="G417" s="13"/>
-      <c r="H417" s="13"/>
-      <c r="I417" s="14" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="J417" s="14" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="K417" s="15"/>
-      <c r="L417" s="15"/>
-      <c r="M417" s="15"/>
-      <c r="N417" s="16"/>
-    </row>
-    <row r="418" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A418" s="12"/>
-      <c r="B418" s="13"/>
-      <c r="C418" s="13"/>
-      <c r="D418" s="13"/>
-      <c r="E418" s="13"/>
-      <c r="F418" s="13"/>
-      <c r="G418" s="13"/>
-      <c r="H418" s="13"/>
-      <c r="I418" s="14" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="J418" s="14" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="K418" s="15"/>
-      <c r="L418" s="15"/>
-      <c r="M418" s="15"/>
-      <c r="N418" s="16"/>
-    </row>
-    <row r="419" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A419" s="12"/>
-      <c r="B419" s="13"/>
-      <c r="C419" s="13"/>
-      <c r="D419" s="13"/>
-      <c r="E419" s="13"/>
-      <c r="F419" s="13"/>
-      <c r="G419" s="13"/>
-      <c r="H419" s="13"/>
-      <c r="I419" s="14" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="J419" s="14" t="str">
-        <f t="shared" si="15"/>
-        <v/>
-      </c>
-      <c r="K419" s="15"/>
-      <c r="L419" s="15"/>
-      <c r="M419" s="15"/>
-      <c r="N419" s="16"/>
-    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A4:N4"/>
@@ -11323,21 +11169,21 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="F3:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="J6:J419">
+  <conditionalFormatting sqref="J6:J412">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K419" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K412" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Excellent,Good,Neutral,Low,Stressed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="L6:L419" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="L6:L412" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Very Satisfied,Satisfied,Neutral,Unsatisfied,Very Unsatisfied"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6:M419" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6:M412" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>